<commit_message>
Hapus nama Rosyid duplikat
</commit_message>
<xml_diff>
--- a/Mufrodat/2. Maret 2026.xlsx
+++ b/Mufrodat/2. Maret 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bahasa-terbaru\Mufrodat\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ASATIDZ\Zen\bahasa-terbaru\Mufrodat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4679FEFD-FB2E-4728-9285-9B59597EFAB7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD68A915-1B94-47AF-9AAB-9FD58E746A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mufrodat" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Mufrodat!$A$1:$C$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Mufrodat Putra'!$A$1:$C$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Mufrodat Putri'!$A$1:$C$48</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Nama Putra'!$A$1:$B$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Nama Putra'!$A$1:$B$33</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Nama Putri'!$A$1:$B$22</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -34,7 +34,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -42,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="173">
   <si>
     <t>Nomor</t>
   </si>
@@ -561,9 +566,6 @@
   </si>
   <si>
     <t>أَمْسِكِي هَذَا قَلِيلًا</t>
-  </si>
-  <si>
-    <t>Rosyid</t>
   </si>
 </sst>
 </file>
@@ -751,12 +753,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -784,7 +780,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1089,11 +1091,11 @@
       <c r="E1" s="26"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
     </row>
     <row r="3" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -1114,7 +1116,7 @@
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="A4" s="24">
         <v>1</v>
       </c>
       <c r="B4" s="13" t="s">
@@ -1131,7 +1133,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="13" t="s">
         <v>102</v>
       </c>
@@ -1147,7 +1149,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="24"/>
       <c r="B6" s="13" t="s">
         <v>61</v>
       </c>
@@ -1163,7 +1165,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="13" t="s">
         <v>62</v>
       </c>
@@ -1179,7 +1181,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="13" t="s">
         <v>63</v>
       </c>
@@ -1195,7 +1197,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
+      <c r="A9" s="25">
         <v>2</v>
       </c>
       <c r="B9" s="12" t="s">
@@ -1207,13 +1209,13 @@
       <c r="D9" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="15">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+      <c r="A10" s="25"/>
       <c r="B10" s="12" t="s">
         <v>103</v>
       </c>
@@ -1223,13 +1225,13 @@
       <c r="D10" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="15">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
+      <c r="A11" s="25"/>
       <c r="B11" s="12" t="s">
         <v>65</v>
       </c>
@@ -1239,13 +1241,13 @@
       <c r="D11" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="15">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+      <c r="A12" s="25"/>
       <c r="B12" s="12" t="s">
         <v>66</v>
       </c>
@@ -1255,13 +1257,13 @@
       <c r="D12" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="15">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+      <c r="A13" s="25"/>
       <c r="B13" s="12" t="s">
         <v>67</v>
       </c>
@@ -1271,13 +1273,13 @@
       <c r="D13" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="24">
         <v>3</v>
       </c>
       <c r="B14" s="13" t="s">
@@ -1295,7 +1297,7 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="13" t="s">
         <v>69</v>
       </c>
@@ -1311,7 +1313,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="13" t="s">
         <v>70</v>
       </c>
@@ -1327,7 +1329,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
+      <c r="A17" s="24"/>
       <c r="B17" s="13" t="s">
         <v>71</v>
       </c>
@@ -1343,7 +1345,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="13" t="s">
         <v>72</v>
       </c>
@@ -1359,7 +1361,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+      <c r="A19" s="25">
         <v>4</v>
       </c>
       <c r="B19" s="12" t="s">
@@ -1371,13 +1373,13 @@
       <c r="D19" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="E19" s="17">
+      <c r="E19" s="15">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
+      <c r="A20" s="25"/>
       <c r="B20" s="12" t="s">
         <v>74</v>
       </c>
@@ -1387,13 +1389,13 @@
       <c r="D20" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="15">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
+      <c r="A21" s="25"/>
       <c r="B21" s="12" t="s">
         <v>75</v>
       </c>
@@ -1403,13 +1405,13 @@
       <c r="D21" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="E21" s="17">
+      <c r="E21" s="15">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
+      <c r="A22" s="25"/>
       <c r="B22" s="12" t="s">
         <v>76</v>
       </c>
@@ -1419,13 +1421,13 @@
       <c r="D22" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="17">
+      <c r="E22" s="15">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
+      <c r="A23" s="25"/>
       <c r="B23" s="12" t="s">
         <v>77</v>
       </c>
@@ -1435,13 +1437,13 @@
       <c r="D23" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="E23" s="17">
+      <c r="E23" s="15">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="24">
         <v>5</v>
       </c>
       <c r="B24" s="13" t="s">
@@ -1459,7 +1461,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="13" t="s">
         <v>79</v>
       </c>
@@ -1475,7 +1477,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="13" t="s">
         <v>80</v>
       </c>
@@ -1491,7 +1493,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="13" t="s">
         <v>81</v>
       </c>
@@ -1507,7 +1509,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="13" t="s">
         <v>82</v>
       </c>
@@ -1523,7 +1525,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16">
+      <c r="A29" s="25">
         <v>6</v>
       </c>
       <c r="B29" s="12" t="s">
@@ -1535,13 +1537,13 @@
       <c r="D29" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="E29" s="17">
+      <c r="E29" s="15">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
+      <c r="A30" s="25"/>
       <c r="B30" s="12" t="s">
         <v>84</v>
       </c>
@@ -1551,13 +1553,13 @@
       <c r="D30" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="E30" s="17">
+      <c r="E30" s="15">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
+      <c r="A31" s="25"/>
       <c r="B31" s="12" t="s">
         <v>85</v>
       </c>
@@ -1567,13 +1569,13 @@
       <c r="D31" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="E31" s="17">
+      <c r="E31" s="15">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
+      <c r="A32" s="25"/>
       <c r="B32" s="12" t="s">
         <v>86</v>
       </c>
@@ -1583,13 +1585,13 @@
       <c r="D32" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="E32" s="17">
+      <c r="E32" s="15">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
+      <c r="A33" s="25"/>
       <c r="B33" s="12" t="s">
         <v>87</v>
       </c>
@@ -1599,13 +1601,13 @@
       <c r="D33" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="E33" s="17">
+      <c r="E33" s="15">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="24">
         <v>7</v>
       </c>
       <c r="B34" s="13" t="s">
@@ -1617,65 +1619,65 @@
       <c r="D34" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="E34" s="21">
+      <c r="E34" s="19">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="15"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="13" t="s">
         <v>89</v>
       </c>
       <c r="C35" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="D35" s="19" t="s">
+      <c r="D35" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="E35" s="22"/>
+      <c r="E35" s="20"/>
     </row>
     <row r="36" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="13" t="s">
         <v>90</v>
       </c>
       <c r="C36" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="D36" s="19" t="s">
+      <c r="D36" s="17" t="s">
         <v>151</v>
       </c>
-      <c r="E36" s="23"/>
+      <c r="E36" s="21"/>
     </row>
     <row r="37" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="15"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="13" t="s">
         <v>91</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="D37" s="19" t="s">
+      <c r="D37" s="17" t="s">
         <v>153</v>
       </c>
-      <c r="E37" s="23"/>
+      <c r="E37" s="21"/>
     </row>
     <row r="38" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="15"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="13" t="s">
         <v>92</v>
       </c>
       <c r="C38" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D38" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="E38" s="23"/>
+      <c r="E38" s="21"/>
     </row>
     <row r="39" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="16">
+      <c r="A39" s="25">
         <v>8</v>
       </c>
       <c r="B39" s="12" t="s">
@@ -1684,65 +1686,65 @@
       <c r="C39" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="D39" s="20" t="s">
+      <c r="D39" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="E39" s="23"/>
+      <c r="E39" s="21"/>
     </row>
     <row r="40" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
+      <c r="A40" s="25"/>
       <c r="B40" s="12" t="s">
         <v>94</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="D40" s="20" t="s">
+      <c r="D40" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="E40" s="23"/>
+      <c r="E40" s="21"/>
     </row>
     <row r="41" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
+      <c r="A41" s="25"/>
       <c r="B41" s="12" t="s">
         <v>95</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="D41" s="20" t="s">
+      <c r="D41" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="E41" s="23"/>
+      <c r="E41" s="21"/>
     </row>
     <row r="42" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+      <c r="A42" s="25"/>
       <c r="B42" s="12" t="s">
         <v>96</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="D42" s="20" t="s">
+      <c r="D42" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="E42" s="23"/>
+      <c r="E42" s="21"/>
     </row>
     <row r="43" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+      <c r="A43" s="25"/>
       <c r="B43" s="12" t="s">
         <v>97</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D43" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="E43" s="23"/>
+      <c r="E43" s="21"/>
     </row>
     <row r="44" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="15">
+      <c r="A44" s="24">
         <v>9</v>
       </c>
       <c r="B44" s="13" t="s">
@@ -1751,65 +1753,66 @@
       <c r="C44" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="D44" s="19" t="s">
+      <c r="D44" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="E44" s="23"/>
+      <c r="E44" s="21"/>
     </row>
     <row r="45" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="13" t="s">
         <v>104</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="D45" s="19" t="s">
+      <c r="D45" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="E45" s="23"/>
+      <c r="E45" s="21"/>
     </row>
     <row r="46" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
+      <c r="A46" s="24"/>
       <c r="B46" s="13" t="s">
         <v>99</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="D46" s="19" t="s">
+      <c r="D46" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="E46" s="23"/>
+      <c r="E46" s="21"/>
     </row>
     <row r="47" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
+      <c r="A47" s="24"/>
       <c r="B47" s="13" t="s">
         <v>100</v>
       </c>
       <c r="C47" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="D47" s="19" t="s">
+      <c r="D47" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="E47" s="23"/>
+      <c r="E47" s="21"/>
     </row>
     <row r="48" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="13" t="s">
         <v>101</v>
       </c>
       <c r="C48" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="D48" s="19" t="s">
+      <c r="D48" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="E48" s="24"/>
+      <c r="E48" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A34:A38"/>
     <mergeCell ref="A39:A43"/>
     <mergeCell ref="A44:A48"/>
@@ -1819,7 +1822,6 @@
     <mergeCell ref="A19:A23"/>
     <mergeCell ref="A24:A28"/>
     <mergeCell ref="A29:A33"/>
-    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0" footer="0"/>
@@ -1849,10 +1851,10 @@
       <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
     </row>
     <row r="3" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -1870,7 +1872,7 @@
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="A4" s="24">
         <v>1</v>
       </c>
       <c r="B4" s="13" t="str">
@@ -1886,7 +1888,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="13" t="str">
         <f>Mufrodat!B5</f>
         <v>Kamu jahat, tidak mau bantuin aku</v>
@@ -1901,7 +1903,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="24"/>
       <c r="B6" s="13" t="str">
         <f>Mufrodat!B6</f>
         <v>Makan lah pakai piring</v>
@@ -1916,7 +1918,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="13" t="str">
         <f>Mufrodat!B7</f>
         <v>Kepalaku pusing bah</v>
@@ -1931,7 +1933,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="13" t="str">
         <f>Mufrodat!B8</f>
         <v>Cepetin bagi makanannya</v>
@@ -1946,84 +1948,84 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
+      <c r="A9" s="25">
         <v>2</v>
       </c>
-      <c r="B9" s="18" t="str">
+      <c r="B9" s="16" t="str">
         <f>Mufrodat!B9</f>
         <v>Apa lauknya?</v>
       </c>
-      <c r="C9" s="18" t="str">
+      <c r="C9" s="16" t="str">
         <f>Mufrodat!C9</f>
         <v>مَا الْإِدَامُ؟</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="15">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="18" t="str">
+      <c r="A10" s="25"/>
+      <c r="B10" s="16" t="str">
         <f>Mufrodat!B10</f>
         <v>Cepetin sudah ada akhwatnya / ikhwannya</v>
       </c>
-      <c r="C10" s="18" t="str">
+      <c r="C10" s="16" t="str">
         <f>Mufrodat!C10</f>
         <v>أَسْرِعْ، فَقَدْ جَاءَتِ الْأَخَوَاتُ</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="15">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="18" t="str">
+      <c r="A11" s="25"/>
+      <c r="B11" s="16" t="str">
         <f>Mufrodat!B11</f>
         <v>Siapa yang piket sapu?</v>
       </c>
-      <c r="C11" s="18" t="str">
+      <c r="C11" s="16" t="str">
         <f>Mufrodat!C11</f>
         <v>مَنْ حَارِسُ الْمَطْعَمِ؟</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="15">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="18" t="str">
+      <c r="A12" s="25"/>
+      <c r="B12" s="16" t="str">
         <f>Mufrodat!B12</f>
         <v>Hijabnya pindah situ</v>
       </c>
-      <c r="C12" s="18" t="str">
+      <c r="C12" s="16" t="str">
         <f>Mufrodat!C12</f>
         <v>اُنْقُلِ الْحِجَابَ إِلَى هُنَاكَ</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="15">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="18" t="str">
+      <c r="A13" s="25"/>
+      <c r="B13" s="16" t="str">
         <f>Mufrodat!B13</f>
         <v>Ah, fresh meat</v>
       </c>
-      <c r="C13" s="18" t="str">
+      <c r="C13" s="16" t="str">
         <f>Mufrodat!C13</f>
         <v>آهِ، لَحْمٌ طَازَجٌ</v>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="24">
         <v>3</v>
       </c>
       <c r="B14" s="13" t="str">
@@ -2040,7 +2042,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="13" t="str">
         <f>Mufrodat!B15</f>
         <v>Jatahku mana?</v>
@@ -2055,7 +2057,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="13" t="str">
         <f>Mufrodat!B16</f>
         <v>Makan apa?</v>
@@ -2070,7 +2072,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
+      <c r="A17" s="24"/>
       <c r="B17" s="13" t="str">
         <f>Mufrodat!B17</f>
         <v>Ambil aja jatahku</v>
@@ -2085,7 +2087,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="13" t="str">
         <f>Mufrodat!B18</f>
         <v>Mana sendok nasi?</v>
@@ -2100,84 +2102,84 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+      <c r="A19" s="25">
         <v>4</v>
       </c>
-      <c r="B19" s="18" t="str">
+      <c r="B19" s="16" t="str">
         <f>Mufrodat!B19</f>
         <v>Kamu nggak makan?</v>
       </c>
-      <c r="C19" s="18" t="str">
+      <c r="C19" s="16" t="str">
         <f>Mufrodat!C19</f>
         <v>أَلَا تَأْكُلُ؟</v>
       </c>
-      <c r="D19" s="17">
+      <c r="D19" s="15">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
-      <c r="B20" s="18" t="str">
+      <c r="A20" s="25"/>
+      <c r="B20" s="16" t="str">
         <f>Mufrodat!B20</f>
         <v>Siapa yang ambil makan?</v>
       </c>
-      <c r="C20" s="18" t="str">
+      <c r="C20" s="16" t="str">
         <f>Mufrodat!C20</f>
         <v>مَنْ أَخَذَ الطَّعَامَ؟</v>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="15">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
-      <c r="B21" s="18" t="str">
+      <c r="A21" s="25"/>
+      <c r="B21" s="16" t="str">
         <f>Mufrodat!B21</f>
         <v>Makannya sudah datang</v>
       </c>
-      <c r="C21" s="18" t="str">
+      <c r="C21" s="16" t="str">
         <f>Mufrodat!C21</f>
         <v>جَاءَ الطَّعَامُ</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="15">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
-      <c r="B22" s="18" t="str">
+      <c r="A22" s="25"/>
+      <c r="B22" s="16" t="str">
         <f>Mufrodat!B22</f>
         <v>Siapa belum makan?</v>
       </c>
-      <c r="C22" s="18" t="str">
+      <c r="C22" s="16" t="str">
         <f>Mufrodat!C22</f>
         <v>مَنْ لَمْ يَأْكُلْ؟</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="15">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="18" t="str">
+      <c r="A23" s="25"/>
+      <c r="B23" s="16" t="str">
         <f>Mufrodat!B23</f>
         <v>Makan di mana?</v>
       </c>
-      <c r="C23" s="18" t="str">
+      <c r="C23" s="16" t="str">
         <f>Mufrodat!C23</f>
         <v>أَيْنَ نَأْكُلُ؟</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="15">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="24">
         <v>5</v>
       </c>
       <c r="B24" s="13" t="str">
@@ -2194,7 +2196,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="13" t="str">
         <f>Mufrodat!B25</f>
         <v>Aku mau makan</v>
@@ -2209,7 +2211,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="13" t="str">
         <f>Mufrodat!B26</f>
         <v>Siapa yang mau makananku?</v>
@@ -2224,7 +2226,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="13" t="str">
         <f>Mufrodat!B27</f>
         <v>Lantainya licin</v>
@@ -2239,7 +2241,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="13" t="str">
         <f>Mufrodat!B28</f>
         <v>Ada sambal kah?</v>
@@ -2254,84 +2256,84 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16">
+      <c r="A29" s="25">
         <v>6</v>
       </c>
-      <c r="B29" s="18" t="str">
+      <c r="B29" s="16" t="str">
         <f>Mufrodat!B29</f>
         <v>Enak betul</v>
       </c>
-      <c r="C29" s="18" t="str">
+      <c r="C29" s="16" t="str">
         <f>Mufrodat!C29</f>
         <v>لَذِيذٌ جِدًّا</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="15">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
-      <c r="B30" s="18" t="str">
+      <c r="A30" s="25"/>
+      <c r="B30" s="16" t="str">
         <f>Mufrodat!B30</f>
         <v>Makan kok masih hamburan</v>
       </c>
-      <c r="C30" s="18" t="str">
+      <c r="C30" s="16" t="str">
         <f>Mufrodat!C30</f>
         <v>لِمَاذَا الطَّعَامُ مُتَنَاثِرٌ هَكَذَا؟</v>
       </c>
-      <c r="D30" s="17">
+      <c r="D30" s="15">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
-      <c r="B31" s="18" t="str">
+      <c r="A31" s="25"/>
+      <c r="B31" s="16" t="str">
         <f>Mufrodat!B31</f>
         <v>Tinggal makan berisik betul</v>
       </c>
-      <c r="C31" s="18" t="str">
+      <c r="C31" s="16" t="str">
         <f>Mufrodat!C31</f>
         <v>الْأَكْلُ فَقَطْ وَمَعَ ذَلِكَ الضَّجِيجُ كَثِيرٌ</v>
       </c>
-      <c r="D31" s="17">
+      <c r="D31" s="15">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
-      <c r="B32" s="18" t="str">
+      <c r="A32" s="25"/>
+      <c r="B32" s="16" t="str">
         <f>Mufrodat!B32</f>
         <v>Awas kepleset</v>
       </c>
-      <c r="C32" s="18" t="str">
+      <c r="C32" s="16" t="str">
         <f>Mufrodat!C32</f>
         <v>اِنْتَبِهْ لَا تَنْزَلِقْ</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="15">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
-      <c r="B33" s="18" t="str">
+      <c r="A33" s="25"/>
+      <c r="B33" s="16" t="str">
         <f>Mufrodat!B33</f>
         <v>Bagi yang rata</v>
       </c>
-      <c r="C33" s="18" t="str">
+      <c r="C33" s="16" t="str">
         <f>Mufrodat!C33</f>
         <v>اِقْسِمْ بِالتَّسَاوِي</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="15">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="24">
         <v>7</v>
       </c>
       <c r="B34" s="13" t="str">
@@ -2342,13 +2344,13 @@
         <f>Mufrodat!C34</f>
         <v>الْإِدَامُ فَاسِدٌ</v>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="19">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="15"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="13" t="str">
         <f>Mufrodat!B35</f>
         <v>Nasinya habis</v>
@@ -2357,10 +2359,10 @@
         <f>Mufrodat!C35</f>
         <v>نَفِدَ الْأَرُزُّ</v>
       </c>
-      <c r="D35" s="22"/>
+      <c r="D35" s="20"/>
     </row>
     <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="13" t="str">
         <f>Mufrodat!B36</f>
         <v>Centongnya tenggelam di bawah nasi</v>
@@ -2369,10 +2371,10 @@
         <f>Mufrodat!C36</f>
         <v>مِغْرَفَةُ الْأَرُزِّ غَارِقَةٌ تَحْتَ الْأَرُزِّ</v>
       </c>
-      <c r="D36" s="23"/>
+      <c r="D36" s="21"/>
     </row>
     <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="15"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="13" t="str">
         <f>Mufrodat!B37</f>
         <v>Siapa yang nggak makan sayur?</v>
@@ -2381,10 +2383,10 @@
         <f>Mufrodat!C37</f>
         <v>مَنْ لَا يَأْكُلُ الْخُضَارَ؟</v>
       </c>
-      <c r="D37" s="23"/>
+      <c r="D37" s="21"/>
     </row>
     <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="15"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="13" t="str">
         <f>Mufrodat!B38</f>
         <v>Nasinya belum matang</v>
@@ -2393,72 +2395,72 @@
         <f>Mufrodat!C38</f>
         <v>الْأَرُزُّ لَمْ يَنْضُجْ بَعْدُ</v>
       </c>
-      <c r="D38" s="23"/>
+      <c r="D38" s="21"/>
     </row>
     <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="16">
+      <c r="A39" s="25">
         <v>8</v>
       </c>
-      <c r="B39" s="18" t="str">
+      <c r="B39" s="16" t="str">
         <f>Mufrodat!B39</f>
         <v>Jangan lama-lama ngambil nasinya</v>
       </c>
-      <c r="C39" s="18" t="str">
+      <c r="C39" s="16" t="str">
         <f>Mufrodat!C39</f>
         <v>لَا تُطِلْ فِي أَخْذِ الْأَرُزِّ</v>
       </c>
-      <c r="D39" s="23"/>
+      <c r="D39" s="21"/>
     </row>
     <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
-      <c r="B40" s="18" t="str">
+      <c r="A40" s="25"/>
+      <c r="B40" s="16" t="str">
         <f>Mufrodat!B40</f>
         <v>Awas licin, baru dipel</v>
       </c>
-      <c r="C40" s="18" t="str">
+      <c r="C40" s="16" t="str">
         <f>Mufrodat!C40</f>
         <v>اِنْتَبِهْ، الْأَرْضُ مَبْلُولَةٌ حَدِيثًا</v>
       </c>
-      <c r="D40" s="23"/>
+      <c r="D40" s="21"/>
     </row>
     <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
-      <c r="B41" s="18" t="str">
+      <c r="A41" s="25"/>
+      <c r="B41" s="16" t="str">
         <f>Mufrodat!B41</f>
         <v>Sendok nasinya masuk parit</v>
       </c>
-      <c r="C41" s="18" t="str">
+      <c r="C41" s="16" t="str">
         <f>Mufrodat!C41</f>
         <v>مِلْعَقَةُ الْأَرُزِّ سَقَطَتْ فِي الْمَجْرَى</v>
       </c>
-      <c r="D41" s="23"/>
+      <c r="D41" s="21"/>
     </row>
     <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
-      <c r="B42" s="18" t="str">
+      <c r="A42" s="25"/>
+      <c r="B42" s="16" t="str">
         <f>Mufrodat!B42</f>
         <v>Tolong, saya keselek sendok</v>
       </c>
-      <c r="C42" s="18" t="str">
+      <c r="C42" s="16" t="str">
         <f>Mufrodat!C42</f>
         <v>سَاعِدْنِي، كِدْتُ أَخْتَنِقُ</v>
       </c>
-      <c r="D42" s="23"/>
+      <c r="D42" s="21"/>
     </row>
     <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
-      <c r="B43" s="18" t="str">
+      <c r="A43" s="25"/>
+      <c r="B43" s="16" t="str">
         <f>Mufrodat!B43</f>
         <v>Jangan loncat, nanti gempa bumi</v>
       </c>
-      <c r="C43" s="18" t="str">
+      <c r="C43" s="16" t="str">
         <f>Mufrodat!C43</f>
         <v>لَا تَقْفِزْ، سَيَحْدُثُ زِلْزَالٌ</v>
       </c>
-      <c r="D43" s="23"/>
+      <c r="D43" s="21"/>
     </row>
     <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="15">
+      <c r="A44" s="24">
         <v>9</v>
       </c>
       <c r="B44" s="13" t="str">
@@ -2469,10 +2471,10 @@
         <f>Mufrodat!C44</f>
         <v>كُلِ التِّمْسَاحَ</v>
       </c>
-      <c r="D44" s="23"/>
+      <c r="D44" s="21"/>
     </row>
     <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="13" t="str">
         <f>Mufrodat!B45</f>
         <v>Minumnya es teh</v>
@@ -2481,10 +2483,10 @@
         <f>Mufrodat!C45</f>
         <v>اِشْرَبْ شَايًا مُثَلَّجًا</v>
       </c>
-      <c r="D45" s="23"/>
+      <c r="D45" s="21"/>
     </row>
     <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
+      <c r="A46" s="24"/>
       <c r="B46" s="13" t="str">
         <f>Mufrodat!B46</f>
         <v>Baksomu di gayung</v>
@@ -2493,10 +2495,10 @@
         <f>Mufrodat!C46</f>
         <v>كُرَاتُ اللَّحْمِ فِي الْمِغْرَفَةِ</v>
       </c>
-      <c r="D46" s="23"/>
+      <c r="D46" s="21"/>
     </row>
     <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
+      <c r="A47" s="24"/>
       <c r="B47" s="13" t="str">
         <f>Mufrodat!B47</f>
         <v>Mau nggak sayurnya?</v>
@@ -2505,10 +2507,10 @@
         <f>Mufrodat!C47</f>
         <v>أَتُرِيدُ الْخُضَارَ؟</v>
       </c>
-      <c r="D47" s="23"/>
+      <c r="D47" s="21"/>
     </row>
     <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="13" t="str">
         <f>Mufrodat!B48</f>
         <v>Titip bentar ya</v>
@@ -2517,7 +2519,7 @@
         <f>Mufrodat!C48</f>
         <v>أَمْسِكْ هَذَا قَلِيلًا</v>
       </c>
-      <c r="D48" s="24"/>
+      <c r="D48" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2534,7 +2536,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="91" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="92" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2560,10 +2562,10 @@
       <c r="D1" s="26"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="A2" s="23"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
     </row>
     <row r="3" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -2581,7 +2583,7 @@
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
+      <c r="A4" s="24">
         <v>1</v>
       </c>
       <c r="B4" s="13" t="str">
@@ -2597,7 +2599,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="13" t="str">
         <f>Mufrodat!B5</f>
         <v>Kamu jahat, tidak mau bantuin aku</v>
@@ -2612,7 +2614,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="24"/>
       <c r="B6" s="13" t="str">
         <f>Mufrodat!B6</f>
         <v>Makan lah pakai piring</v>
@@ -2627,7 +2629,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="13" t="str">
         <f>Mufrodat!B7</f>
         <v>Kepalaku pusing bah</v>
@@ -2642,7 +2644,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
+      <c r="A8" s="24"/>
       <c r="B8" s="13" t="str">
         <f>Mufrodat!B8</f>
         <v>Cepetin bagi makanannya</v>
@@ -2657,84 +2659,84 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16">
+      <c r="A9" s="25">
         <v>2</v>
       </c>
-      <c r="B9" s="18" t="str">
+      <c r="B9" s="16" t="str">
         <f>Mufrodat!B9</f>
         <v>Apa lauknya?</v>
       </c>
-      <c r="C9" s="18" t="str">
+      <c r="C9" s="16" t="str">
         <f>Mufrodat!D9</f>
         <v>مَا الْإِدَامُ؟</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="15">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="18" t="str">
+      <c r="A10" s="25"/>
+      <c r="B10" s="16" t="str">
         <f>Mufrodat!B10</f>
         <v>Cepetin sudah ada akhwatnya / ikhwannya</v>
       </c>
-      <c r="C10" s="18" t="str">
+      <c r="C10" s="16" t="str">
         <f>Mufrodat!D10</f>
         <v>أَسْرِعِي، فَقَدْ جَاءَ الْإِخْوَانُ</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="15">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="18" t="str">
+      <c r="A11" s="25"/>
+      <c r="B11" s="16" t="str">
         <f>Mufrodat!B11</f>
         <v>Siapa yang piket sapu?</v>
       </c>
-      <c r="C11" s="18" t="str">
+      <c r="C11" s="16" t="str">
         <f>Mufrodat!D11</f>
         <v>مَنْ حَارِسَةُ الْمَطْعَمِ؟</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="15">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="18" t="str">
+      <c r="A12" s="25"/>
+      <c r="B12" s="16" t="str">
         <f>Mufrodat!B12</f>
         <v>Hijabnya pindah situ</v>
       </c>
-      <c r="C12" s="18" t="str">
+      <c r="C12" s="16" t="str">
         <f>Mufrodat!D12</f>
         <v>اُنْقُلِي الْحِجَابَ إِلَى هُنَاكِ</v>
       </c>
-      <c r="D12" s="17">
+      <c r="D12" s="15">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="18" t="str">
+      <c r="A13" s="25"/>
+      <c r="B13" s="16" t="str">
         <f>Mufrodat!B13</f>
         <v>Ah, fresh meat</v>
       </c>
-      <c r="C13" s="18" t="str">
+      <c r="C13" s="16" t="str">
         <f>Mufrodat!D13</f>
         <v>آهِ، لَحْمٌ طَازَجٌ</v>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
+      <c r="A14" s="24">
         <v>3</v>
       </c>
       <c r="B14" s="13" t="str">
@@ -2751,7 +2753,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
+      <c r="A15" s="24"/>
       <c r="B15" s="13" t="str">
         <f>Mufrodat!B15</f>
         <v>Jatahku mana?</v>
@@ -2766,7 +2768,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
+      <c r="A16" s="24"/>
       <c r="B16" s="13" t="str">
         <f>Mufrodat!B16</f>
         <v>Makan apa?</v>
@@ -2781,7 +2783,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
+      <c r="A17" s="24"/>
       <c r="B17" s="13" t="str">
         <f>Mufrodat!B17</f>
         <v>Ambil aja jatahku</v>
@@ -2796,7 +2798,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
+      <c r="A18" s="24"/>
       <c r="B18" s="13" t="str">
         <f>Mufrodat!B18</f>
         <v>Mana sendok nasi?</v>
@@ -2811,84 +2813,84 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16">
+      <c r="A19" s="25">
         <v>4</v>
       </c>
-      <c r="B19" s="18" t="str">
+      <c r="B19" s="16" t="str">
         <f>Mufrodat!B19</f>
         <v>Kamu nggak makan?</v>
       </c>
-      <c r="C19" s="18" t="str">
+      <c r="C19" s="16" t="str">
         <f>Mufrodat!D19</f>
         <v>أَلَا تَأْكُلِينَ؟</v>
       </c>
-      <c r="D19" s="17">
+      <c r="D19" s="15">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
-      <c r="B20" s="18" t="str">
+      <c r="A20" s="25"/>
+      <c r="B20" s="16" t="str">
         <f>Mufrodat!B20</f>
         <v>Siapa yang ambil makan?</v>
       </c>
-      <c r="C20" s="18" t="str">
+      <c r="C20" s="16" t="str">
         <f>Mufrodat!D20</f>
         <v>مَنْ أَخَذَ الطَّعَامَ؟</v>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="15">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
-      <c r="B21" s="18" t="str">
+      <c r="A21" s="25"/>
+      <c r="B21" s="16" t="str">
         <f>Mufrodat!B21</f>
         <v>Makannya sudah datang</v>
       </c>
-      <c r="C21" s="18" t="str">
+      <c r="C21" s="16" t="str">
         <f>Mufrodat!D21</f>
         <v>جَاءَ الطَّعَامُ</v>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="15">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
-      <c r="B22" s="18" t="str">
+      <c r="A22" s="25"/>
+      <c r="B22" s="16" t="str">
         <f>Mufrodat!B22</f>
         <v>Siapa belum makan?</v>
       </c>
-      <c r="C22" s="18" t="str">
+      <c r="C22" s="16" t="str">
         <f>Mufrodat!D22</f>
         <v>مَنْ لَمْ تَأْكُلْ؟</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="15">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="18" t="str">
+      <c r="A23" s="25"/>
+      <c r="B23" s="16" t="str">
         <f>Mufrodat!B23</f>
         <v>Makan di mana?</v>
       </c>
-      <c r="C23" s="18" t="str">
+      <c r="C23" s="16" t="str">
         <f>Mufrodat!D23</f>
         <v>أَيْنَ نَأْكُلُ؟</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="15">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
+      <c r="A24" s="24">
         <v>5</v>
       </c>
       <c r="B24" s="13" t="str">
@@ -2905,7 +2907,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
+      <c r="A25" s="24"/>
       <c r="B25" s="13" t="str">
         <f>Mufrodat!B25</f>
         <v>Aku mau makan</v>
@@ -2920,7 +2922,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
+      <c r="A26" s="24"/>
       <c r="B26" s="13" t="str">
         <f>Mufrodat!B26</f>
         <v>Siapa yang mau makananku?</v>
@@ -2935,7 +2937,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
+      <c r="A27" s="24"/>
       <c r="B27" s="13" t="str">
         <f>Mufrodat!B27</f>
         <v>Lantainya licin</v>
@@ -2950,7 +2952,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
+      <c r="A28" s="24"/>
       <c r="B28" s="13" t="str">
         <f>Mufrodat!B28</f>
         <v>Ada sambal kah?</v>
@@ -2965,84 +2967,84 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16">
+      <c r="A29" s="25">
         <v>6</v>
       </c>
-      <c r="B29" s="18" t="str">
+      <c r="B29" s="16" t="str">
         <f>Mufrodat!B29</f>
         <v>Enak betul</v>
       </c>
-      <c r="C29" s="18" t="str">
+      <c r="C29" s="16" t="str">
         <f>Mufrodat!D29</f>
         <v>لَذِيذٌ جِدًّا</v>
       </c>
-      <c r="D29" s="17">
+      <c r="D29" s="15">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
-      <c r="B30" s="18" t="str">
+      <c r="A30" s="25"/>
+      <c r="B30" s="16" t="str">
         <f>Mufrodat!B30</f>
         <v>Makan kok masih hamburan</v>
       </c>
-      <c r="C30" s="18" t="str">
+      <c r="C30" s="16" t="str">
         <f>Mufrodat!D30</f>
         <v>لِمَاذَا الطَّعَامُ مُتَنَاثِرٌ هَكَذَا؟</v>
       </c>
-      <c r="D30" s="17">
+      <c r="D30" s="15">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
-      <c r="B31" s="18" t="str">
+      <c r="A31" s="25"/>
+      <c r="B31" s="16" t="str">
         <f>Mufrodat!B31</f>
         <v>Tinggal makan berisik betul</v>
       </c>
-      <c r="C31" s="18" t="str">
+      <c r="C31" s="16" t="str">
         <f>Mufrodat!D31</f>
         <v>الْأَكْلُ فَقَطْ وَمَعَ ذَلِكَ الضَّجِيجُ كَثِيرٌ</v>
       </c>
-      <c r="D31" s="17">
+      <c r="D31" s="15">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
-      <c r="B32" s="18" t="str">
+      <c r="A32" s="25"/>
+      <c r="B32" s="16" t="str">
         <f>Mufrodat!B32</f>
         <v>Awas kepleset</v>
       </c>
-      <c r="C32" s="18" t="str">
+      <c r="C32" s="16" t="str">
         <f>Mufrodat!D32</f>
         <v>اِنْتَبِهِي لَا تَنْزَلِقِي</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="15">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
-      <c r="B33" s="18" t="str">
+      <c r="A33" s="25"/>
+      <c r="B33" s="16" t="str">
         <f>Mufrodat!B33</f>
         <v>Bagi yang rata</v>
       </c>
-      <c r="C33" s="18" t="str">
+      <c r="C33" s="16" t="str">
         <f>Mufrodat!D33</f>
         <v>اِقْسِمِي بِالتَّسَاوِي</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="15">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
+      <c r="A34" s="24">
         <v>7</v>
       </c>
       <c r="B34" s="13" t="str">
@@ -3053,13 +3055,13 @@
         <f>Mufrodat!D34</f>
         <v>الْإِدَامُ فَاسِدٌ</v>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="19">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="15"/>
+      <c r="A35" s="24"/>
       <c r="B35" s="13" t="str">
         <f>Mufrodat!B35</f>
         <v>Nasinya habis</v>
@@ -3068,10 +3070,10 @@
         <f>Mufrodat!D35</f>
         <v>نَفِدَ الْأَرُزُّ</v>
       </c>
-      <c r="D35" s="22"/>
+      <c r="D35" s="20"/>
     </row>
     <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
+      <c r="A36" s="24"/>
       <c r="B36" s="13" t="str">
         <f>Mufrodat!B36</f>
         <v>Centongnya tenggelam di bawah nasi</v>
@@ -3080,10 +3082,10 @@
         <f>Mufrodat!D36</f>
         <v>مِغْرَفَةُ الْأَرُزِّ غَارِقَةٌ تَحْتَ الْأَرُزِّ</v>
       </c>
-      <c r="D36" s="23"/>
+      <c r="D36" s="21"/>
     </row>
     <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="15"/>
+      <c r="A37" s="24"/>
       <c r="B37" s="13" t="str">
         <f>Mufrodat!B37</f>
         <v>Siapa yang nggak makan sayur?</v>
@@ -3092,10 +3094,10 @@
         <f>Mufrodat!D37</f>
         <v>مَنْ لَا تَأْكُلُ الْخُضَارَ؟</v>
       </c>
-      <c r="D37" s="23"/>
+      <c r="D37" s="21"/>
     </row>
     <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="15"/>
+      <c r="A38" s="24"/>
       <c r="B38" s="13" t="str">
         <f>Mufrodat!B38</f>
         <v>Nasinya belum matang</v>
@@ -3104,72 +3106,72 @@
         <f>Mufrodat!D38</f>
         <v>الْأَرُزُّ لَمْ يَنْضُجْ بَعْدُ</v>
       </c>
-      <c r="D38" s="23"/>
+      <c r="D38" s="21"/>
     </row>
     <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="16">
+      <c r="A39" s="25">
         <v>8</v>
       </c>
-      <c r="B39" s="18" t="str">
+      <c r="B39" s="16" t="str">
         <f>Mufrodat!B39</f>
         <v>Jangan lama-lama ngambil nasinya</v>
       </c>
-      <c r="C39" s="18" t="str">
+      <c r="C39" s="16" t="str">
         <f>Mufrodat!D39</f>
         <v>لَا تُطِيلِي فِي أَخْذِ الْأَرُزِّ</v>
       </c>
-      <c r="D39" s="23"/>
+      <c r="D39" s="21"/>
     </row>
     <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
-      <c r="B40" s="18" t="str">
+      <c r="A40" s="25"/>
+      <c r="B40" s="16" t="str">
         <f>Mufrodat!B40</f>
         <v>Awas licin, baru dipel</v>
       </c>
-      <c r="C40" s="18" t="str">
+      <c r="C40" s="16" t="str">
         <f>Mufrodat!D40</f>
         <v>اِنْتَبِهِي، الْأَرْضُ مَبْلُولَةٌ حَدِيثًا</v>
       </c>
-      <c r="D40" s="23"/>
+      <c r="D40" s="21"/>
     </row>
     <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16"/>
-      <c r="B41" s="18" t="str">
+      <c r="A41" s="25"/>
+      <c r="B41" s="16" t="str">
         <f>Mufrodat!B41</f>
         <v>Sendok nasinya masuk parit</v>
       </c>
-      <c r="C41" s="18" t="str">
+      <c r="C41" s="16" t="str">
         <f>Mufrodat!D41</f>
         <v>مِلْعَقَةُ الْأَرُزِّ سَقَطَتْ فِي الْمَجْرَى</v>
       </c>
-      <c r="D41" s="23"/>
+      <c r="D41" s="21"/>
     </row>
     <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
-      <c r="B42" s="18" t="str">
+      <c r="A42" s="25"/>
+      <c r="B42" s="16" t="str">
         <f>Mufrodat!B42</f>
         <v>Tolong, saya keselek sendok</v>
       </c>
-      <c r="C42" s="18" t="str">
+      <c r="C42" s="16" t="str">
         <f>Mufrodat!D42</f>
         <v>سَاعِدِينِي، كِدْتُ أَخْتَنِقُ</v>
       </c>
-      <c r="D42" s="23"/>
+      <c r="D42" s="21"/>
     </row>
     <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
-      <c r="B43" s="18" t="str">
+      <c r="A43" s="25"/>
+      <c r="B43" s="16" t="str">
         <f>Mufrodat!B43</f>
         <v>Jangan loncat, nanti gempa bumi</v>
       </c>
-      <c r="C43" s="18" t="str">
+      <c r="C43" s="16" t="str">
         <f>Mufrodat!D43</f>
         <v>لَا تَقْفِزِي، سَيَحْدُثُ زِلْزَالٌ</v>
       </c>
-      <c r="D43" s="23"/>
+      <c r="D43" s="21"/>
     </row>
     <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="15">
+      <c r="A44" s="24">
         <v>9</v>
       </c>
       <c r="B44" s="13" t="str">
@@ -3180,10 +3182,10 @@
         <f>Mufrodat!D44</f>
         <v>كُلِي التِّمْسَاحَ</v>
       </c>
-      <c r="D44" s="23"/>
+      <c r="D44" s="21"/>
     </row>
     <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
+      <c r="A45" s="24"/>
       <c r="B45" s="13" t="str">
         <f>Mufrodat!B45</f>
         <v>Minumnya es teh</v>
@@ -3192,10 +3194,10 @@
         <f>Mufrodat!D45</f>
         <v>اِشْرَبِي شَايًا مُثَلَّجًا</v>
       </c>
-      <c r="D45" s="23"/>
+      <c r="D45" s="21"/>
     </row>
     <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
+      <c r="A46" s="24"/>
       <c r="B46" s="13" t="str">
         <f>Mufrodat!B46</f>
         <v>Baksomu di gayung</v>
@@ -3204,10 +3206,10 @@
         <f>Mufrodat!D46</f>
         <v>كُرَاتُ اللَّحْمِ فِي الْمِغْرَفَةِ</v>
       </c>
-      <c r="D46" s="23"/>
+      <c r="D46" s="21"/>
     </row>
     <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
+      <c r="A47" s="24"/>
       <c r="B47" s="13" t="str">
         <f>Mufrodat!B47</f>
         <v>Mau nggak sayurnya?</v>
@@ -3216,10 +3218,10 @@
         <f>Mufrodat!D47</f>
         <v>أَتُرِيدِينَ الْخُضَارَ؟</v>
       </c>
-      <c r="D47" s="23"/>
+      <c r="D47" s="21"/>
     </row>
     <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
+      <c r="A48" s="24"/>
       <c r="B48" s="13" t="str">
         <f>Mufrodat!B48</f>
         <v>Titip bentar ya</v>
@@ -3228,7 +3230,7 @@
         <f>Mufrodat!D48</f>
         <v>أَمْسِكِي هَذَا قَلِيلًا</v>
       </c>
-      <c r="D48" s="24"/>
+      <c r="D48" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -3245,7 +3247,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="91" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="92" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3254,7 +3256,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
@@ -3532,14 +3534,6 @@
       </c>
       <c r="B33" s="7" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
-        <v>6</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>